<commit_message>
feat(api_tel): add ListarUnidades class for fetching and processing TJSP unit data
- Implemented methods to retrieve and process forum units based on municipality codes.
- Utilized concurrent requests for improved performance.
- Added properties for accessing processed data, including municipalities and comarcas.
- Integrated BeautifulSoup for HTML parsing and data extraction.
</commit_message>
<xml_diff>
--- a/data/output/tab/Comarcas e CJs.xlsx
+++ b/data/output/tab/Comarcas e CJs.xlsx
@@ -431,7 +431,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adamantina </t>
+          <t>Adamantina</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -441,7 +441,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aguaí </t>
+          <t>Aguaí</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -451,7 +451,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Agudos </t>
+          <t>Agudos</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -461,7 +461,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Altinópolis </t>
+          <t>Altinópolis</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -471,7 +471,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Americana </t>
+          <t>Americana</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -481,7 +481,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Américo Brasiliense </t>
+          <t>Américo Brasiliense</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -491,7 +491,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Amparo </t>
+          <t>Amparo</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -501,7 +501,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Andradina </t>
+          <t>Andradina</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -511,7 +511,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Angatuba </t>
+          <t>Angatuba</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -521,7 +521,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aparecida </t>
+          <t>Aparecida</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -531,7 +531,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apiaí </t>
+          <t>Apiaí</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -541,7 +541,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Araçatuba </t>
+          <t>Araçatuba</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -551,7 +551,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Araraquara </t>
+          <t>Araraquara</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -561,7 +561,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Araras </t>
+          <t>Araras</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -571,7 +571,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artur Nogueira </t>
+          <t>Artur Nogueira</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -581,7 +581,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arujá </t>
+          <t>Arujá</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -591,7 +591,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assis </t>
+          <t>Assis</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -601,7 +601,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Atibaia </t>
+          <t>Atibaia</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -611,7 +611,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auriflama </t>
+          <t>Auriflama</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -621,7 +621,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Avaré </t>
+          <t>Avaré</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -631,7 +631,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Águas de Lindóia </t>
+          <t>Águas de Lindóia</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -641,7 +641,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bananal </t>
+          <t>Bananal</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -651,7 +651,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bariri </t>
+          <t>Bariri</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -661,7 +661,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Barra Bonita </t>
+          <t>Barra Bonita</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -671,7 +671,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Barretos </t>
+          <t>Barretos</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -681,7 +681,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Barueri </t>
+          <t>Barueri</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -691,7 +691,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bastos </t>
+          <t>Bastos</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -701,7 +701,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Batatais </t>
+          <t>Batatais</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -711,7 +711,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bauru </t>
+          <t>Bauru</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -721,7 +721,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bebedouro </t>
+          <t>Bebedouro</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -731,7 +731,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bertioga </t>
+          <t>Bertioga</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -741,7 +741,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bilac </t>
+          <t>Bilac</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -751,7 +751,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Birigui </t>
+          <t>Birigui</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -761,7 +761,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boituva </t>
+          <t>Boituva</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -771,7 +771,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Borborema </t>
+          <t>Borborema</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -781,7 +781,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Botucatu </t>
+          <t>Botucatu</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -791,7 +791,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bragança Paulista </t>
+          <t>Bragança Paulista</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -801,7 +801,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brodowski </t>
+          <t>Brodowski</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -811,7 +811,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brotas </t>
+          <t>Brotas</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -821,7 +821,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buri </t>
+          <t>Buri</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -831,7 +831,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buritama </t>
+          <t>Buritama</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -841,7 +841,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cabreúva </t>
+          <t>Cabreúva</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -851,7 +851,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cachoeira Paulista </t>
+          <t>Cachoeira Paulista</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -861,7 +861,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caconde </t>
+          <t>Caconde</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -871,7 +871,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caçapava </t>
+          <t>Caçapava</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -881,7 +881,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cafelândia </t>
+          <t>Cafelândia</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -891,7 +891,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caieiras </t>
+          <t>Caieiras</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -901,7 +901,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cajamar </t>
+          <t>Cajamar</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -911,7 +911,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cajuru </t>
+          <t>Cajuru</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -921,7 +921,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Campinas </t>
+          <t>Campinas</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -931,7 +931,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Campo Limpo Paulista </t>
+          <t>Campo Limpo Paulista</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -941,7 +941,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Campos do Jordão </t>
+          <t>Campos do Jordão</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -951,7 +951,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cananéia </t>
+          <t>Cananéia</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -961,7 +961,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capão Bonito </t>
+          <t>Capão Bonito</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -971,7 +971,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capivari </t>
+          <t>Capivari</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -981,7 +981,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caraguatatuba </t>
+          <t>Caraguatatuba</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -991,7 +991,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carapicuiba </t>
+          <t>Carapicuiba</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1001,7 +1001,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cardoso </t>
+          <t>Cardoso</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1011,7 +1011,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Casa Branca </t>
+          <t>Casa Branca</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1021,7 +1021,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Catanduva </t>
+          <t>Catanduva</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1031,7 +1031,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cândido Mota </t>
+          <t>Cândido Mota</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1041,7 +1041,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cerqueira Cesar </t>
+          <t>Cerqueira Cesar</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1051,7 +1051,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cerquilho </t>
+          <t>Cerquilho</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1061,7 +1061,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cesário Lange </t>
+          <t>Cesário Lange</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1071,7 +1071,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chavantes </t>
+          <t>Chavantes</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1081,7 +1081,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Colina </t>
+          <t>Colina</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1091,7 +1091,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conchal </t>
+          <t>Conchal</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1101,7 +1101,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conchas </t>
+          <t>Conchas</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1111,7 +1111,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cordeirópolis </t>
+          <t>Cordeirópolis</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1121,7 +1121,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cosmópolis </t>
+          <t>Cosmópolis</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1131,7 +1131,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cotia </t>
+          <t>Cotia</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1141,7 +1141,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cravinhos </t>
+          <t>Cravinhos</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1151,7 +1151,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cruzeiro </t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1161,7 +1161,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cubatão </t>
+          <t>Cubatão</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1171,7 +1171,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cunha </t>
+          <t>Cunha</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1181,7 +1181,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Descalvado </t>
+          <t>Descalvado</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1191,7 +1191,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diadema </t>
+          <t>Diadema</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1201,7 +1201,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dois Córregos </t>
+          <t>Dois Córregos</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1211,7 +1211,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dracena </t>
+          <t>Dracena</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1221,7 +1221,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Duartina </t>
+          <t>Duartina</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1231,7 +1231,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eldorado </t>
+          <t>Eldorado</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1241,7 +1241,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Embu das Artes </t>
+          <t>Embu das Artes</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1251,7 +1251,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Embu-Guaçu </t>
+          <t>Embu-Guaçu</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1261,7 +1261,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Espírito Santo do Pinhal </t>
+          <t>Espírito Santo do Pinhal</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1271,7 +1271,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estrela D’Oeste </t>
+          <t>Estrela D’Oeste</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1281,7 +1281,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fartura </t>
+          <t>Fartura</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1291,7 +1291,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fernandópolis </t>
+          <t>Fernandópolis</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1301,7 +1301,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ferraz de Vasconcelos </t>
+          <t>Ferraz de Vasconcelos</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1311,7 +1311,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flórida Paulista </t>
+          <t>Flórida Paulista</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1321,7 +1321,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Franca </t>
+          <t>Franca</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1331,7 +1331,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Francisco Morato </t>
+          <t>Francisco Morato</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1341,7 +1341,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Franco da Rocha </t>
+          <t>Franco da Rocha</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1351,7 +1351,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Garça </t>
+          <t>Garça</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1361,7 +1361,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gália </t>
+          <t>Gália</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1371,7 +1371,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">General Salgado </t>
+          <t>General Salgado</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1381,7 +1381,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Getulina </t>
+          <t>Getulina</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1391,7 +1391,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guaíra </t>
+          <t>Guaíra</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1401,7 +1401,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guararapes </t>
+          <t>Guararapes</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -1411,7 +1411,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guararema </t>
+          <t>Guararema</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -1421,7 +1421,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guaratinguetá </t>
+          <t>Guaratinguetá</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -1431,7 +1431,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guará </t>
+          <t>Guará</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -1441,7 +1441,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guariba </t>
+          <t>Guariba</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -1451,7 +1451,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guarujá </t>
+          <t>Guarujá</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -1461,7 +1461,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guarulhos </t>
+          <t>Guarulhos</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -1471,7 +1471,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hortolândia </t>
+          <t>Hortolândia</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -1481,7 +1481,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iacanga </t>
+          <t>Iacanga</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -1491,7 +1491,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ibaté </t>
+          <t>Ibaté</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -1501,7 +1501,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ibitinga </t>
+          <t>Ibitinga</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -1511,7 +1511,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ibiúna </t>
+          <t>Ibiúna</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -1521,7 +1521,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iepê </t>
+          <t>Iepê</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -1531,7 +1531,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Igarapava </t>
+          <t>Igarapava</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -1541,7 +1541,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iguape </t>
+          <t>Iguape</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -1551,7 +1551,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ilha Solteira </t>
+          <t>Ilha Solteira</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -1561,7 +1561,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ilhabela </t>
+          <t>Ilhabela</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -1571,7 +1571,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indaiatuba </t>
+          <t>Indaiatuba</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -1581,7 +1581,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ipaussu </t>
+          <t>Ipaussu</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -1591,7 +1591,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ipuã </t>
+          <t>Ipuã</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -1601,7 +1601,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itaberá </t>
+          <t>Itaberá</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -1611,7 +1611,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itaí </t>
+          <t>Itaí</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -1621,7 +1621,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itajobi </t>
+          <t>Itajobi</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -1631,7 +1631,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itanhaém </t>
+          <t>Itanhaém</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -1641,7 +1641,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itapecerica da Serra </t>
+          <t>Itapecerica da Serra</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -1651,7 +1651,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itapetininga </t>
+          <t>Itapetininga</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -1661,7 +1661,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itapeva </t>
+          <t>Itapeva</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -1671,7 +1671,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itapevi </t>
+          <t>Itapevi</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -1681,7 +1681,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itapira </t>
+          <t>Itapira</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -1691,7 +1691,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itaporanga </t>
+          <t>Itaporanga</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -1701,7 +1701,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itaquaquecetuba </t>
+          <t>Itaquaquecetuba</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -1711,7 +1711,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itararé </t>
+          <t>Itararé</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -1721,7 +1721,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itariri </t>
+          <t>Itariri</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -1731,7 +1731,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itatiba </t>
+          <t>Itatiba</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -1741,7 +1741,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itatinga </t>
+          <t>Itatinga</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -1751,7 +1751,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itápolis </t>
+          <t>Itápolis</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -1761,7 +1761,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itirapina </t>
+          <t>Itirapina</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -1771,7 +1771,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itu </t>
+          <t>Itu</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -1781,7 +1781,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Itupeva </t>
+          <t>Itupeva</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -1791,7 +1791,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ituverava </t>
+          <t>Ituverava</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -1801,7 +1801,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jaboticabal </t>
+          <t>Jaboticabal</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -1811,7 +1811,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jacareí </t>
+          <t>Jacareí</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -1821,7 +1821,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jacupiranga </t>
+          <t>Jacupiranga</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -1831,7 +1831,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jaguariúna </t>
+          <t>Jaguariúna</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -1841,7 +1841,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jales </t>
+          <t>Jales</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -1851,7 +1851,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jandira </t>
+          <t>Jandira</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -1861,7 +1861,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jardinópolis </t>
+          <t>Jardinópolis</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -1871,7 +1871,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jarinu </t>
+          <t>Jarinu</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -1881,7 +1881,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jaú </t>
+          <t>Jaú</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -1891,7 +1891,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">José Bonifácio </t>
+          <t>José Bonifácio</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -1901,7 +1901,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jundiaí </t>
+          <t>Jundiaí</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -1911,7 +1911,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Junqueirópolis </t>
+          <t>Junqueirópolis</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -1921,7 +1921,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Juquiá </t>
+          <t>Juquiá</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -1931,7 +1931,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laranjal Paulista </t>
+          <t>Laranjal Paulista</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -1941,7 +1941,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leme </t>
+          <t>Leme</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -1951,7 +1951,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lençóis Paulista </t>
+          <t>Lençóis Paulista</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -1961,7 +1961,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Limeira </t>
+          <t>Limeira</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -1971,7 +1971,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lins </t>
+          <t>Lins</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -1981,7 +1981,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lorena </t>
+          <t>Lorena</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -1991,7 +1991,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Louveira </t>
+          <t>Louveira</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2001,7 +2001,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lucélia </t>
+          <t>Lucélia</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2011,7 +2011,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Macatuba </t>
+          <t>Macatuba</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2021,7 +2021,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Macaubal </t>
+          <t>Macaubal</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -2031,7 +2031,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mairinque </t>
+          <t>Mairinque</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -2041,7 +2041,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mairiporã </t>
+          <t>Mairiporã</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -2051,7 +2051,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maracaí </t>
+          <t>Maracaí</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -2061,7 +2061,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marília </t>
+          <t>Marília</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -2071,7 +2071,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t xml:space="preserve">Martinópolis </t>
+          <t>Martinópolis</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -2081,7 +2081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t xml:space="preserve">Matão </t>
+          <t>Matão</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -2091,7 +2091,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mauá </t>
+          <t>Mauá</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -2101,7 +2101,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miguelópolis </t>
+          <t>Miguelópolis</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -2111,7 +2111,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miracatu </t>
+          <t>Miracatu</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -2121,7 +2121,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mirandópolis </t>
+          <t>Mirandópolis</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -2131,7 +2131,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mirante do Paranapanema </t>
+          <t>Mirante do Paranapanema</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -2141,7 +2141,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mirassol </t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -2151,7 +2151,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mococa </t>
+          <t>Mococa</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -2161,7 +2161,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mogi Guaçu </t>
+          <t>Mogi Guaçu</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -2171,7 +2171,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mogi Mirim </t>
+          <t>Mogi Mirim</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -2181,7 +2181,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mogi das Cruzes </t>
+          <t>Mogi das Cruzes</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -2191,7 +2191,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mongaguá </t>
+          <t>Mongaguá</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -2201,7 +2201,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monte Alto </t>
+          <t>Monte Alto</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -2211,7 +2211,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monte Aprazível </t>
+          <t>Monte Aprazível</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -2221,7 +2221,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monte Azul Paulista </t>
+          <t>Monte Azul Paulista</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -2231,7 +2231,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monte Mor </t>
+          <t>Monte Mor</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -2241,7 +2241,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Morro Agudo </t>
+          <t>Morro Agudo</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -2251,7 +2251,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nazaré Paulista </t>
+          <t>Nazaré Paulista</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -2261,7 +2261,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t xml:space="preserve">Neves Paulista </t>
+          <t>Neves Paulista</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -2271,7 +2271,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhandeara </t>
+          <t>Nhandeara</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -2281,7 +2281,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nova Granada </t>
+          <t>Nova Granada</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -2291,7 +2291,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nova Odessa </t>
+          <t>Nova Odessa</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -2301,7 +2301,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">Novo Horizonte </t>
+          <t>Novo Horizonte</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -2311,7 +2311,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nuporanga </t>
+          <t>Nuporanga</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -2321,7 +2321,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t xml:space="preserve">Olímpia </t>
+          <t>Olímpia</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -2331,7 +2331,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Orlândia </t>
+          <t>Orlândia</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -2341,7 +2341,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Osasco </t>
+          <t>Osasco</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -2351,7 +2351,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Osvaldo Cruz </t>
+          <t>Osvaldo Cruz</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -2361,7 +2361,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ourinhos </t>
+          <t>Ourinhos</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -2371,7 +2371,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ouroeste </t>
+          <t>Ouroeste</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -2381,7 +2381,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pacaembu </t>
+          <t>Pacaembu</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -2391,7 +2391,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Palestina </t>
+          <t>Palestina</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -2401,7 +2401,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t xml:space="preserve">Palmeira D’Oeste </t>
+          <t>Palmeira D’Oeste</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -2411,7 +2411,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Palmital </t>
+          <t>Palmital</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -2421,7 +2421,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Panorama </t>
+          <t>Panorama</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -2431,7 +2431,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paraguaçu Paulista </t>
+          <t>Paraguaçu Paulista</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -2441,7 +2441,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paraibuna </t>
+          <t>Paraibuna</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -2451,7 +2451,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paranapanema </t>
+          <t>Paranapanema</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -2461,7 +2461,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pariquera-Açu </t>
+          <t>Pariquera-Açu</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -2471,7 +2471,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrocínio Paulista </t>
+          <t>Patrocínio Paulista</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -2481,7 +2481,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paulínia </t>
+          <t>Paulínia</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -2491,7 +2491,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paulo de Faria </t>
+          <t>Paulo de Faria</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -2501,7 +2501,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pederneiras </t>
+          <t>Pederneiras</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -2511,7 +2511,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pedregulho </t>
+          <t>Pedregulho</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -2521,7 +2521,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pedreira </t>
+          <t>Pedreira</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -2531,7 +2531,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t xml:space="preserve">Penápolis </t>
+          <t>Penápolis</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -2541,7 +2541,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pereira Barreto </t>
+          <t>Pereira Barreto</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -2551,7 +2551,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peruíbe </t>
+          <t>Peruíbe</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -2561,7 +2561,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Piedade </t>
+          <t>Piedade</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -2571,7 +2571,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilar do Sul </t>
+          <t>Pilar do Sul</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -2581,7 +2581,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pindamonhangaba </t>
+          <t>Pindamonhangaba</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -2591,7 +2591,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pinhalzinho </t>
+          <t>Pinhalzinho</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -2601,7 +2601,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Piquete </t>
+          <t>Piquete</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -2611,7 +2611,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Piracaia </t>
+          <t>Piracaia</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -2621,7 +2621,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Piracicaba </t>
+          <t>Piracicaba</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -2631,7 +2631,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Piraju </t>
+          <t>Piraju</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -2641,7 +2641,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pirajuí </t>
+          <t>Pirajuí</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -2651,7 +2651,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pirangi </t>
+          <t>Pirangi</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -2661,7 +2661,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pirapozinho </t>
+          <t>Pirapozinho</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -2671,7 +2671,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pirassununga </t>
+          <t>Pirassununga</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -2681,7 +2681,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Piratininga </t>
+          <t>Piratininga</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -2691,7 +2691,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pitangueiras </t>
+          <t>Pitangueiras</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -2701,7 +2701,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poá </t>
+          <t>Poá</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -2711,7 +2711,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pompéia </t>
+          <t>Pompéia</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -2721,7 +2721,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pontal </t>
+          <t>Pontal</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -2731,7 +2731,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Porangaba </t>
+          <t>Porangaba</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -2741,7 +2741,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Porto Feliz </t>
+          <t>Porto Feliz</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -2751,7 +2751,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Porto Ferreira </t>
+          <t>Porto Ferreira</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -2761,7 +2761,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Potirendaba </t>
+          <t>Potirendaba</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -2771,7 +2771,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t xml:space="preserve">Praia Grande </t>
+          <t>Praia Grande</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -2781,7 +2781,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presidente Bernardes </t>
+          <t>Presidente Bernardes</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -2791,7 +2791,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presidente Epitácio </t>
+          <t>Presidente Epitácio</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -2801,7 +2801,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presidente Prudente </t>
+          <t>Presidente Prudente</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -2811,7 +2811,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presidente Venceslau </t>
+          <t>Presidente Venceslau</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -2821,7 +2821,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Promissão </t>
+          <t>Promissão</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -2831,7 +2831,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quatá </t>
+          <t>Quatá</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -2841,7 +2841,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Queluz </t>
+          <t>Queluz</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -2851,7 +2851,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rancharia </t>
+          <t>Rancharia</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -2861,7 +2861,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Regente Feijó </t>
+          <t>Regente Feijó</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -2871,7 +2871,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registro </t>
+          <t>Registro</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -2881,7 +2881,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ribeirão Bonito </t>
+          <t>Ribeirão Bonito</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -2891,7 +2891,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ribeirão Pires </t>
+          <t>Ribeirão Pires</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -2901,7 +2901,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ribeirão Preto </t>
+          <t>Ribeirão Preto</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -2911,7 +2911,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rio Claro </t>
+          <t>Rio Claro</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -2921,7 +2921,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rio Grande de Serra </t>
+          <t>Rio Grande de Serra</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -2931,7 +2931,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rio das Pedras </t>
+          <t>Rio das Pedras</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -2941,7 +2941,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rosana </t>
+          <t>Rosana</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -2951,7 +2951,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Roseira </t>
+          <t>Roseira</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -2961,7 +2961,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Salesópolis </t>
+          <t>Salesópolis</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -2971,7 +2971,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Salto </t>
+          <t>Salto</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -2981,7 +2981,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Salto de Pirapora </t>
+          <t>Salto de Pirapora</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -2991,7 +2991,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santa Adélia </t>
+          <t>Santa Adélia</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -3001,7 +3001,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santa Bárbara D’Oeste </t>
+          <t>Santa Bárbara D’Oeste</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -3011,7 +3011,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santa Branca </t>
+          <t>Santa Branca</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -3021,7 +3021,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santa Cruz das Palmeiras </t>
+          <t>Santa Cruz das Palmeiras</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -3031,7 +3031,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santa Cruz do Rio Pardo </t>
+          <t>Santa Cruz do Rio Pardo</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -3041,7 +3041,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santa Fé do Sul </t>
+          <t>Santa Fé do Sul</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -3051,7 +3051,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santa Isabel </t>
+          <t>Santa Isabel</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -3061,7 +3061,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santa Rita do Passa Quatro </t>
+          <t>Santa Rita do Passa Quatro</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -3071,7 +3071,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santa Rosa do Viterbo </t>
+          <t>Santa Rosa do Viterbo</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -3081,7 +3081,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santana do Parnaíba </t>
+          <t>Santana do Parnaíba</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -3091,7 +3091,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santo Anastácio </t>
+          <t>Santo Anastácio</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -3101,7 +3101,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santo André </t>
+          <t>Santo André</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -3111,7 +3111,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t xml:space="preserve">Santos </t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -3121,7 +3121,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Bento do Sapucaí </t>
+          <t>São Bento do Sapucaí</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -3131,7 +3131,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Bernardo do Campo </t>
+          <t>São Bernardo do Campo</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -3141,7 +3141,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Caetano do Sul </t>
+          <t>São Caetano do Sul</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -3151,7 +3151,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Carlos </t>
+          <t>São Carlos</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -3161,7 +3161,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Joaquim da Barra </t>
+          <t>São Joaquim da Barra</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -3171,7 +3171,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t xml:space="preserve">São João da Boa Vista </t>
+          <t>São João da Boa Vista</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -3181,7 +3181,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t xml:space="preserve">São José do Rio Pardo </t>
+          <t>São José do Rio Pardo</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -3191,7 +3191,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t xml:space="preserve">São José do Rio Preto </t>
+          <t>São José do Rio Preto</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -3201,7 +3201,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t xml:space="preserve">São José dos Campos </t>
+          <t>São José dos Campos</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -3211,7 +3211,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Luis do Paraitinga </t>
+          <t>São Luis do Paraitinga</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -3221,7 +3221,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Manuel </t>
+          <t>São Manuel</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -3231,7 +3231,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Miguel Arcanjo </t>
+          <t>São Miguel Arcanjo</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -3241,7 +3241,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Paulo </t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -3251,7 +3251,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Pedro </t>
+          <t>São Pedro</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -3261,7 +3261,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Roque </t>
+          <t>São Roque</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -3271,7 +3271,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Sebastião </t>
+          <t>São Sebastião</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -3281,7 +3281,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Sebastião da Grama </t>
+          <t>São Sebastião da Grama</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -3291,7 +3291,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Simão </t>
+          <t>São Simão</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -3301,7 +3301,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t xml:space="preserve">São Vicente </t>
+          <t>São Vicente</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -3311,7 +3311,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t xml:space="preserve">Serra Negra </t>
+          <t>Serra Negra</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -3321,7 +3321,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t xml:space="preserve">Serrana </t>
+          <t>Serrana</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -3331,7 +3331,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sertãozinho </t>
+          <t>Sertãozinho</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -3341,7 +3341,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t xml:space="preserve">Socorro </t>
+          <t>Socorro</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -3351,7 +3351,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sorocaba </t>
+          <t>Sorocaba</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -3361,7 +3361,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sumaré </t>
+          <t>Sumaré</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -3371,7 +3371,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suzano </t>
+          <t>Suzano</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -3381,7 +3381,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tabapuã </t>
+          <t>Tabapuã</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -3391,7 +3391,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t xml:space="preserve">Taboão da Serra </t>
+          <t>Taboão da Serra</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -3401,7 +3401,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tambaú </t>
+          <t>Tambaú</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -3411,7 +3411,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tanabi </t>
+          <t>Tanabi</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -3421,7 +3421,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t xml:space="preserve">Taquaritinga </t>
+          <t>Taquaritinga</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -3431,7 +3431,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t xml:space="preserve">Taquarituba </t>
+          <t>Taquarituba</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -3441,7 +3441,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tatuí </t>
+          <t>Tatuí</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -3451,7 +3451,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t xml:space="preserve">Taubaté </t>
+          <t>Taubaté</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -3461,7 +3461,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teodoro Sampaio </t>
+          <t>Teodoro Sampaio</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -3471,7 +3471,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tietê </t>
+          <t>Tietê</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -3481,7 +3481,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tremembé </t>
+          <t>Tremembé</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -3491,7 +3491,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tupã </t>
+          <t>Tupã</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -3501,7 +3501,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tupi Paulista </t>
+          <t>Tupi Paulista</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -3511,7 +3511,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ubatuba </t>
+          <t>Ubatuba</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -3521,7 +3521,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t xml:space="preserve">Urânia </t>
+          <t>Urânia</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -3531,7 +3531,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t xml:space="preserve">Urupês </t>
+          <t>Urupês</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -3541,7 +3541,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valinhos </t>
+          <t>Valinhos</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -3551,7 +3551,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -3561,7 +3561,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vargem Grande Paulista </t>
+          <t>Vargem Grande Paulista</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -3571,7 +3571,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vargem Grande do Sul </t>
+          <t>Vargem Grande do Sul</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -3581,7 +3581,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t xml:space="preserve">Várzea Paulista </t>
+          <t>Várzea Paulista</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -3591,7 +3591,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vila Mimosa </t>
+          <t>Vila Mimosa</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -3601,7 +3601,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vinhedo </t>
+          <t>Vinhedo</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -3611,7 +3611,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t xml:space="preserve">Viradouro </t>
+          <t>Viradouro</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -3621,7 +3621,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t xml:space="preserve">Votorantim </t>
+          <t>Votorantim</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -3631,7 +3631,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t xml:space="preserve">Votuporanga </t>
+          <t>Votuporanga</t>
         </is>
       </c>
       <c r="B322" t="n">

</xml_diff>